<commit_message>
fix(dry-run): stop the lifecycle sheets carrying the Act 5 reprice
Pat confirmed on 2026-07-31 that a published line never moves, so the
close/open/final sheets should not inherit the +110 -> -140 reprice.

They were derived from `repriced`, which meant skipping the optional Act 5
upload did not skip the reprice: 2-phase1-closed-r1-results.xlsx carried the
new line and would have shortened Dan Mercer silently during the close.

Sheets 2-4 now derive from phase1Open. 1b-phase1-repriced.xlsx is still
generated for anyone exercising the odds-snapshot rule deliberately.

Payouts are unaffected either way -- lib/payouts.ts reads odds_at_placement,
never the live pick.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/dry-run/sheets/2-phase1-closed-r1-results.xlsx
+++ b/docs/dry-run/sheets/2-phase1-closed-r1-results.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="95">
   <si>
     <t>phase</t>
   </si>
@@ -73,7 +73,7 @@
     <t>Dan Mercer</t>
   </si>
   <si>
-    <t>7/12</t>
+    <t>11/10</t>
   </si>
   <si>
     <t>Hit</t>
@@ -164,9 +164,6 @@
   </si>
   <si>
     <t>Medalist - Round 1</t>
-  </si>
-  <si>
-    <t>11/10</t>
   </si>
   <si>
     <t>6/1</t>
@@ -755,16 +752,16 @@
         <v>19</v>
       </c>
       <c r="I2">
-        <v>-140</v>
+        <v>110</v>
       </c>
       <c r="J2" t="s">
         <v>20</v>
       </c>
       <c r="K2">
-        <v>0.5833333333333334</v>
+        <v>0.47619047619047616</v>
       </c>
       <c r="L2">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M2" t="s">
         <v>21</v>
@@ -805,7 +802,7 @@
         <v>0.3333333333333333</v>
       </c>
       <c r="L3">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M3" t="s">
         <v>24</v>
@@ -846,7 +843,7 @@
         <v>0.2</v>
       </c>
       <c r="L4">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M4" t="s">
         <v>24</v>
@@ -887,7 +884,7 @@
         <v>0.1</v>
       </c>
       <c r="L5">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M5" t="s">
         <v>24</v>
@@ -928,7 +925,7 @@
         <v>0.125</v>
       </c>
       <c r="L6">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M6" t="s">
         <v>24</v>
@@ -969,7 +966,7 @@
         <v>0.07692307692307693</v>
       </c>
       <c r="L7">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M7" t="s">
         <v>24</v>
@@ -1010,7 +1007,7 @@
         <v>0.0625</v>
       </c>
       <c r="L8">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M8" t="s">
         <v>24</v>
@@ -1051,7 +1048,7 @@
         <v>0.0625</v>
       </c>
       <c r="L9">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M9" t="s">
         <v>24</v>
@@ -1092,7 +1089,7 @@
         <v>0.0625</v>
       </c>
       <c r="L10">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M10" t="s">
         <v>24</v>
@@ -1133,7 +1130,7 @@
         <v>0.0196078431372549</v>
       </c>
       <c r="L11">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M11" t="s">
         <v>24</v>
@@ -1174,7 +1171,7 @@
         <v>0.0196078431372549</v>
       </c>
       <c r="L12">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M12" t="s">
         <v>24</v>
@@ -1215,7 +1212,7 @@
         <v>0.009900990099009901</v>
       </c>
       <c r="L13">
-        <v>1.6552064199632632</v>
+        <v>1.548063562820406</v>
       </c>
       <c r="M13" t="s">
         <v>24</v>
@@ -1660,7 +1657,7 @@
         <v>110</v>
       </c>
       <c r="J24" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="K24">
         <v>0.47619047619047616</v>
@@ -1783,7 +1780,7 @@
         <v>600</v>
       </c>
       <c r="J27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K27">
         <v>0.14285714285714285</v>
@@ -1824,7 +1821,7 @@
         <v>600</v>
       </c>
       <c r="J28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="K28">
         <v>0.14285714285714285</v>
@@ -2134,7 +2131,7 @@
         <v>49</v>
       </c>
       <c r="D36" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E36">
         <v>4</v>
@@ -2143,7 +2140,7 @@
         <v>35</v>
       </c>
       <c r="G36" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H36" t="s">
         <v>19</v>
@@ -2152,7 +2149,7 @@
         <v>-130</v>
       </c>
       <c r="J36" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K36">
         <v>0.5652173913043478</v>
@@ -2175,7 +2172,7 @@
         <v>49</v>
       </c>
       <c r="D37" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E37">
         <v>4</v>
@@ -2184,7 +2181,7 @@
         <v>36</v>
       </c>
       <c r="G37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H37" t="s">
         <v>22</v>
@@ -2193,7 +2190,7 @@
         <v>130</v>
       </c>
       <c r="J37" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K37">
         <v>0.43478260869565216</v>
@@ -2216,7 +2213,7 @@
         <v>49</v>
       </c>
       <c r="D38" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E38">
         <v>5</v>
@@ -2225,7 +2222,7 @@
         <v>37</v>
       </c>
       <c r="G38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H38" t="s">
         <v>25</v>
@@ -2257,7 +2254,7 @@
         <v>49</v>
       </c>
       <c r="D39" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E39">
         <v>5</v>
@@ -2266,7 +2263,7 @@
         <v>38</v>
       </c>
       <c r="G39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H39" t="s">
         <v>27</v>
@@ -2275,7 +2272,7 @@
         <v>250</v>
       </c>
       <c r="J39" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K39">
         <v>0.2857142857142857</v>
@@ -2298,7 +2295,7 @@
         <v>49</v>
       </c>
       <c r="D40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E40">
         <v>5</v>
@@ -2307,7 +2304,7 @@
         <v>39</v>
       </c>
       <c r="G40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H40" t="s">
         <v>29</v>
@@ -2339,7 +2336,7 @@
         <v>49</v>
       </c>
       <c r="D41" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E41">
         <v>5</v>
@@ -2348,7 +2345,7 @@
         <v>40</v>
       </c>
       <c r="G41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H41" t="s">
         <v>31</v>
@@ -2380,7 +2377,7 @@
         <v>49</v>
       </c>
       <c r="D42" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E42">
         <v>6</v>
@@ -2389,7 +2386,7 @@
         <v>41</v>
       </c>
       <c r="G42" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H42" t="s">
         <v>35</v>
@@ -2407,7 +2404,7 @@
         <v>1</v>
       </c>
       <c r="M42" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
@@ -2421,7 +2418,7 @@
         <v>49</v>
       </c>
       <c r="D43" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E43">
         <v>6</v>
@@ -2430,7 +2427,7 @@
         <v>42</v>
       </c>
       <c r="G43" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H43" t="s">
         <v>36</v>
@@ -2448,7 +2445,7 @@
         <v>1</v>
       </c>
       <c r="M43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
@@ -2462,7 +2459,7 @@
         <v>49</v>
       </c>
       <c r="D44" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E44">
         <v>7</v>
@@ -2471,10 +2468,10 @@
         <v>43</v>
       </c>
       <c r="G44" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H44" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I44">
         <v>150</v>
@@ -2503,7 +2500,7 @@
         <v>49</v>
       </c>
       <c r="D45" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E45">
         <v>7</v>
@@ -2512,10 +2509,10 @@
         <v>44</v>
       </c>
       <c r="G45" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H45" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I45">
         <v>150</v>
@@ -2544,7 +2541,7 @@
         <v>49</v>
       </c>
       <c r="D46" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E46">
         <v>7</v>
@@ -2553,10 +2550,10 @@
         <v>45</v>
       </c>
       <c r="G46" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="H46" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I46">
         <v>150</v>
@@ -2585,7 +2582,7 @@
         <v>49</v>
       </c>
       <c r="D47" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E47">
         <v>8</v>
@@ -2594,10 +2591,10 @@
         <v>46</v>
       </c>
       <c r="G47" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H47" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I47">
         <v>100</v>
@@ -2612,7 +2609,7 @@
         <v>1</v>
       </c>
       <c r="M47" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
@@ -2626,7 +2623,7 @@
         <v>49</v>
       </c>
       <c r="D48" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E48">
         <v>8</v>
@@ -2635,10 +2632,10 @@
         <v>47</v>
       </c>
       <c r="G48" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="H48" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I48">
         <v>100</v>
@@ -2653,7 +2650,7 @@
         <v>1</v>
       </c>
       <c r="M48" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
@@ -2667,7 +2664,7 @@
         <v>49</v>
       </c>
       <c r="D49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E49">
         <v>9</v>
@@ -2676,10 +2673,10 @@
         <v>48</v>
       </c>
       <c r="G49" t="s">
+        <v>67</v>
+      </c>
+      <c r="H49" t="s">
         <v>68</v>
-      </c>
-      <c r="H49" t="s">
-        <v>69</v>
       </c>
       <c r="I49">
         <v>200</v>
@@ -2708,7 +2705,7 @@
         <v>49</v>
       </c>
       <c r="D50" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E50">
         <v>9</v>
@@ -2717,16 +2714,16 @@
         <v>49</v>
       </c>
       <c r="G50" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H50" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I50">
         <v>-200</v>
       </c>
       <c r="J50" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K50">
         <v>0.6666666666666666</v>
@@ -2749,7 +2746,7 @@
         <v>49</v>
       </c>
       <c r="D51" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E51">
         <v>10</v>
@@ -2758,10 +2755,10 @@
         <v>50</v>
       </c>
       <c r="G51" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H51" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I51">
         <v>150</v>
@@ -2790,7 +2787,7 @@
         <v>49</v>
       </c>
       <c r="D52" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E52">
         <v>10</v>
@@ -2799,16 +2796,16 @@
         <v>51</v>
       </c>
       <c r="G52" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="H52" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I52">
         <v>-150</v>
       </c>
       <c r="J52" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="K52">
         <v>0.6</v>
@@ -2831,7 +2828,7 @@
         <v>49</v>
       </c>
       <c r="D53" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E53">
         <v>11</v>
@@ -2840,16 +2837,16 @@
         <v>52</v>
       </c>
       <c r="G53" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H53" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I53">
         <v>-130</v>
       </c>
       <c r="J53" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K53">
         <v>0.5652173913043478</v>
@@ -2858,7 +2855,7 @@
         <v>1</v>
       </c>
       <c r="M53" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="54" spans="1:15" x14ac:dyDescent="0.25">
@@ -2872,7 +2869,7 @@
         <v>49</v>
       </c>
       <c r="D54" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E54">
         <v>11</v>
@@ -2881,16 +2878,16 @@
         <v>53</v>
       </c>
       <c r="G54" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H54" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I54">
         <v>130</v>
       </c>
       <c r="J54" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K54">
         <v>0.43478260869565216</v>
@@ -2899,7 +2896,7 @@
         <v>1</v>
       </c>
       <c r="M54" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="55" spans="1:15" x14ac:dyDescent="0.25">
@@ -2913,7 +2910,7 @@
         <v>49</v>
       </c>
       <c r="D55" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E55">
         <v>12</v>
@@ -2922,16 +2919,16 @@
         <v>54</v>
       </c>
       <c r="G55" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H55" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I55">
         <v>-110</v>
       </c>
       <c r="J55" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="K55">
         <v>0.5238095238095238</v>
@@ -2954,7 +2951,7 @@
         <v>49</v>
       </c>
       <c r="D56" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E56">
         <v>12</v>
@@ -2963,16 +2960,16 @@
         <v>55</v>
       </c>
       <c r="G56" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H56" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I56">
         <v>110</v>
       </c>
       <c r="J56" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="K56">
         <v>0.47619047619047616</v>
@@ -2995,7 +2992,7 @@
         <v>49</v>
       </c>
       <c r="D57" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E57">
         <v>13</v>
@@ -3004,16 +3001,16 @@
         <v>56</v>
       </c>
       <c r="G57" t="s">
+        <v>76</v>
+      </c>
+      <c r="H57" t="s">
         <v>77</v>
-      </c>
-      <c r="H57" t="s">
-        <v>78</v>
       </c>
       <c r="I57">
         <v>-120</v>
       </c>
       <c r="J57" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K57">
         <v>0.5454545454545454</v>
@@ -3036,7 +3033,7 @@
         <v>49</v>
       </c>
       <c r="D58" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E58">
         <v>13</v>
@@ -3045,16 +3042,16 @@
         <v>57</v>
       </c>
       <c r="G58" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H58" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I58">
         <v>120</v>
       </c>
       <c r="J58" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K58">
         <v>0.45454545454545453</v>
@@ -3071,7 +3068,7 @@
         <v>2</v>
       </c>
       <c r="B59" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C59" t="s">
         <v>16</v>
@@ -3104,7 +3101,7 @@
         <v>1.2575757575757576</v>
       </c>
       <c r="M59" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.25">
@@ -3112,7 +3109,7 @@
         <v>2</v>
       </c>
       <c r="B60" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C60" t="s">
         <v>16</v>
@@ -3136,7 +3133,7 @@
         <v>250</v>
       </c>
       <c r="J60" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K60">
         <v>0.2857142857142857</v>
@@ -3145,7 +3142,7 @@
         <v>1.2575757575757576</v>
       </c>
       <c r="M60" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.25">
@@ -3153,7 +3150,7 @@
         <v>2</v>
       </c>
       <c r="B61" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C61" t="s">
         <v>16</v>
@@ -3186,7 +3183,7 @@
         <v>1.2575757575757576</v>
       </c>
       <c r="M61" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.25">
@@ -3194,7 +3191,7 @@
         <v>2</v>
       </c>
       <c r="B62" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C62" t="s">
         <v>16</v>
@@ -3218,7 +3215,7 @@
         <v>1000</v>
       </c>
       <c r="J62" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K62">
         <v>0.09090909090909091</v>
@@ -3227,7 +3224,7 @@
         <v>1.2575757575757576</v>
       </c>
       <c r="M62" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.25">
@@ -3235,7 +3232,7 @@
         <v>2</v>
       </c>
       <c r="B63" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C63" t="s">
         <v>16</v>
@@ -3259,7 +3256,7 @@
         <v>2000</v>
       </c>
       <c r="J63" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="K63">
         <v>0.047619047619047616</v>
@@ -3268,7 +3265,7 @@
         <v>1.2575757575757576</v>
       </c>
       <c r="M63" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
@@ -3276,7 +3273,7 @@
         <v>2</v>
       </c>
       <c r="B64" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C64" t="s">
         <v>16</v>
@@ -3291,7 +3288,7 @@
         <v>63</v>
       </c>
       <c r="G64" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H64" t="s">
         <v>36</v>
@@ -3300,7 +3297,7 @@
         <v>120</v>
       </c>
       <c r="J64" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K64">
         <v>0.45454545454545453</v>
@@ -3309,7 +3306,7 @@
         <v>2.311942959001782</v>
       </c>
       <c r="M64" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.25">
@@ -3317,7 +3314,7 @@
         <v>2</v>
       </c>
       <c r="B65" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C65" t="s">
         <v>16</v>
@@ -3332,7 +3329,7 @@
         <v>64</v>
       </c>
       <c r="G65" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H65" t="s">
         <v>27</v>
@@ -3341,7 +3338,7 @@
         <v>120</v>
       </c>
       <c r="J65" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K65">
         <v>0.45454545454545453</v>
@@ -3350,7 +3347,7 @@
         <v>2.311942959001782</v>
       </c>
       <c r="M65" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="66" spans="1:15" x14ac:dyDescent="0.25">
@@ -3358,7 +3355,7 @@
         <v>2</v>
       </c>
       <c r="B66" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C66" t="s">
         <v>16</v>
@@ -3373,7 +3370,7 @@
         <v>65</v>
       </c>
       <c r="G66" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H66" t="s">
         <v>33</v>
@@ -3382,7 +3379,7 @@
         <v>120</v>
       </c>
       <c r="J66" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K66">
         <v>0.45454545454545453</v>
@@ -3391,7 +3388,7 @@
         <v>2.311942959001782</v>
       </c>
       <c r="M66" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="67" spans="1:15" x14ac:dyDescent="0.25">
@@ -3399,7 +3396,7 @@
         <v>2</v>
       </c>
       <c r="B67" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C67" t="s">
         <v>16</v>
@@ -3414,10 +3411,10 @@
         <v>66</v>
       </c>
       <c r="G67" t="s">
+        <v>85</v>
+      </c>
+      <c r="H67" t="s">
         <v>86</v>
-      </c>
-      <c r="H67" t="s">
-        <v>87</v>
       </c>
       <c r="I67">
         <v>5000</v>
@@ -3432,7 +3429,7 @@
         <v>2.311942959001782</v>
       </c>
       <c r="M67" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="68" spans="1:15" x14ac:dyDescent="0.25">
@@ -3440,7 +3437,7 @@
         <v>2</v>
       </c>
       <c r="B68" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C68" t="s">
         <v>16</v>
@@ -3455,7 +3452,7 @@
         <v>67</v>
       </c>
       <c r="G68" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H68" t="s">
         <v>31</v>
@@ -3464,7 +3461,7 @@
         <v>120</v>
       </c>
       <c r="J68" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K68">
         <v>0.45454545454545453</v>
@@ -3473,7 +3470,7 @@
         <v>2.311942959001782</v>
       </c>
       <c r="M68" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="69" spans="1:15" x14ac:dyDescent="0.25">
@@ -3481,7 +3478,7 @@
         <v>2</v>
       </c>
       <c r="B69" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C69" t="s">
         <v>16</v>
@@ -3496,7 +3493,7 @@
         <v>68</v>
       </c>
       <c r="G69" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H69" t="s">
         <v>35</v>
@@ -3505,7 +3502,7 @@
         <v>120</v>
       </c>
       <c r="J69" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K69">
         <v>0.45454545454545453</v>
@@ -3514,7 +3511,7 @@
         <v>2.311942959001782</v>
       </c>
       <c r="M69" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="70" spans="1:15" x14ac:dyDescent="0.25">
@@ -3522,7 +3519,7 @@
         <v>2</v>
       </c>
       <c r="B70" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C70" t="s">
         <v>16</v>
@@ -3537,7 +3534,7 @@
         <v>69</v>
       </c>
       <c r="G70" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="H70" t="s">
         <v>40</v>
@@ -3555,7 +3552,7 @@
         <v>2.311942959001782</v>
       </c>
       <c r="M70" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="71" spans="1:15" x14ac:dyDescent="0.25">
@@ -3563,10 +3560,10 @@
         <v>2</v>
       </c>
       <c r="B71" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C71" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D71" t="s">
         <v>17</v>
@@ -3578,7 +3575,7 @@
         <v>70</v>
       </c>
       <c r="G71" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H71" t="s">
         <v>19</v>
@@ -3587,7 +3584,7 @@
         <v>110</v>
       </c>
       <c r="J71" t="s">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="K71">
         <v>0.47619047619047616</v>
@@ -3596,7 +3593,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M71" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.25">
@@ -3604,10 +3601,10 @@
         <v>2</v>
       </c>
       <c r="B72" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C72" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D72" t="s">
         <v>17</v>
@@ -3619,7 +3616,7 @@
         <v>71</v>
       </c>
       <c r="G72" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H72" t="s">
         <v>22</v>
@@ -3628,7 +3625,7 @@
         <v>120</v>
       </c>
       <c r="J72" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K72">
         <v>0.45454545454545453</v>
@@ -3637,7 +3634,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M72" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.25">
@@ -3645,10 +3642,10 @@
         <v>2</v>
       </c>
       <c r="B73" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C73" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D73" t="s">
         <v>17</v>
@@ -3660,7 +3657,7 @@
         <v>72</v>
       </c>
       <c r="G73" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H73" t="s">
         <v>25</v>
@@ -3669,7 +3666,7 @@
         <v>220</v>
       </c>
       <c r="J73" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="K73">
         <v>0.3125</v>
@@ -3678,7 +3675,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M73" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="74" spans="1:15" x14ac:dyDescent="0.25">
@@ -3686,10 +3683,10 @@
         <v>2</v>
       </c>
       <c r="B74" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C74" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D74" t="s">
         <v>17</v>
@@ -3701,7 +3698,7 @@
         <v>73</v>
       </c>
       <c r="G74" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H74" t="s">
         <v>27</v>
@@ -3710,7 +3707,7 @@
         <v>1000</v>
       </c>
       <c r="J74" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="K74">
         <v>0.09090909090909091</v>
@@ -3719,7 +3716,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M74" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="75" spans="1:15" x14ac:dyDescent="0.25">
@@ -3727,10 +3724,10 @@
         <v>2</v>
       </c>
       <c r="B75" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C75" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D75" t="s">
         <v>17</v>
@@ -3742,7 +3739,7 @@
         <v>74</v>
       </c>
       <c r="G75" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H75" t="s">
         <v>29</v>
@@ -3760,7 +3757,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M75" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="76" spans="1:15" x14ac:dyDescent="0.25">
@@ -3768,10 +3765,10 @@
         <v>2</v>
       </c>
       <c r="B76" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C76" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D76" t="s">
         <v>17</v>
@@ -3783,7 +3780,7 @@
         <v>75</v>
       </c>
       <c r="G76" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H76" t="s">
         <v>31</v>
@@ -3801,7 +3798,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M76" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="77" spans="1:15" x14ac:dyDescent="0.25">
@@ -3809,10 +3806,10 @@
         <v>2</v>
       </c>
       <c r="B77" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C77" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D77" t="s">
         <v>17</v>
@@ -3824,7 +3821,7 @@
         <v>76</v>
       </c>
       <c r="G77" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H77" t="s">
         <v>33</v>
@@ -3842,7 +3839,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M77" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="78" spans="1:15" x14ac:dyDescent="0.25">
@@ -3850,10 +3847,10 @@
         <v>2</v>
       </c>
       <c r="B78" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C78" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D78" t="s">
         <v>17</v>
@@ -3865,7 +3862,7 @@
         <v>77</v>
       </c>
       <c r="G78" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H78" t="s">
         <v>35</v>
@@ -3883,7 +3880,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M78" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="79" spans="1:15" x14ac:dyDescent="0.25">
@@ -3891,10 +3888,10 @@
         <v>2</v>
       </c>
       <c r="B79" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C79" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D79" t="s">
         <v>17</v>
@@ -3906,7 +3903,7 @@
         <v>78</v>
       </c>
       <c r="G79" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H79" t="s">
         <v>36</v>
@@ -3924,7 +3921,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M79" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="80" spans="1:15" x14ac:dyDescent="0.25">
@@ -3932,10 +3929,10 @@
         <v>2</v>
       </c>
       <c r="B80" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C80" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D80" t="s">
         <v>17</v>
@@ -3947,7 +3944,7 @@
         <v>79</v>
       </c>
       <c r="G80" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H80" t="s">
         <v>37</v>
@@ -3965,7 +3962,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M80" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="81" spans="1:15" x14ac:dyDescent="0.25">
@@ -3973,10 +3970,10 @@
         <v>2</v>
       </c>
       <c r="B81" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C81" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D81" t="s">
         <v>17</v>
@@ -3988,7 +3985,7 @@
         <v>80</v>
       </c>
       <c r="G81" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H81" t="s">
         <v>39</v>
@@ -4006,7 +4003,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M81" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="82" spans="1:15" x14ac:dyDescent="0.25">
@@ -4014,10 +4011,10 @@
         <v>2</v>
       </c>
       <c r="B82" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C82" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D82" t="s">
         <v>17</v>
@@ -4029,7 +4026,7 @@
         <v>81</v>
       </c>
       <c r="G82" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H82" t="s">
         <v>40</v>
@@ -4047,7 +4044,7 @@
         <v>1.7246078518646948</v>
       </c>
       <c r="M82" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="83" spans="1:15" x14ac:dyDescent="0.25">
@@ -4055,13 +4052,13 @@
         <v>2</v>
       </c>
       <c r="B83" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C83" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D83" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E83">
         <v>17</v>
@@ -4070,10 +4067,10 @@
         <v>82</v>
       </c>
       <c r="G83" t="s">
+        <v>90</v>
+      </c>
+      <c r="H83" t="s">
         <v>91</v>
-      </c>
-      <c r="H83" t="s">
-        <v>92</v>
       </c>
       <c r="I83">
         <v>100</v>
@@ -4088,7 +4085,7 @@
         <v>1</v>
       </c>
       <c r="M83" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="84" spans="1:15" x14ac:dyDescent="0.25">
@@ -4096,13 +4093,13 @@
         <v>2</v>
       </c>
       <c r="B84" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C84" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D84" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E84">
         <v>17</v>
@@ -4111,10 +4108,10 @@
         <v>83</v>
       </c>
       <c r="G84" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H84" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I84">
         <v>100</v>
@@ -4129,7 +4126,7 @@
         <v>1</v>
       </c>
       <c r="M84" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="85" spans="1:15" x14ac:dyDescent="0.25">
@@ -4137,13 +4134,13 @@
         <v>2</v>
       </c>
       <c r="B85" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C85" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D85" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E85">
         <v>18</v>
@@ -4152,10 +4149,10 @@
         <v>84</v>
       </c>
       <c r="G85" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H85" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I85">
         <v>100</v>
@@ -4170,7 +4167,7 @@
         <v>1</v>
       </c>
       <c r="M85" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="86" spans="1:15" x14ac:dyDescent="0.25">
@@ -4178,13 +4175,13 @@
         <v>2</v>
       </c>
       <c r="B86" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C86" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D86" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E86">
         <v>18</v>
@@ -4193,10 +4190,10 @@
         <v>85</v>
       </c>
       <c r="G86" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H86" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="I86">
         <v>100</v>
@@ -4211,7 +4208,7 @@
         <v>1</v>
       </c>
       <c r="M86" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="87" spans="1:15" x14ac:dyDescent="0.25">
@@ -4219,13 +4216,13 @@
         <v>2</v>
       </c>
       <c r="B87" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C87" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D87" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E87">
         <v>19</v>
@@ -4234,16 +4231,16 @@
         <v>86</v>
       </c>
       <c r="G87" t="s">
+        <v>76</v>
+      </c>
+      <c r="H87" t="s">
         <v>77</v>
-      </c>
-      <c r="H87" t="s">
-        <v>78</v>
       </c>
       <c r="I87">
         <v>-120</v>
       </c>
       <c r="J87" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K87">
         <v>0.5454545454545454</v>
@@ -4252,7 +4249,7 @@
         <v>1</v>
       </c>
       <c r="M87" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="88" spans="1:15" x14ac:dyDescent="0.25">
@@ -4260,13 +4257,13 @@
         <v>2</v>
       </c>
       <c r="B88" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C88" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D88" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E88">
         <v>19</v>
@@ -4275,16 +4272,16 @@
         <v>87</v>
       </c>
       <c r="G88" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H88" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="I88">
         <v>120</v>
       </c>
       <c r="J88" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K88">
         <v>0.45454545454545453</v>
@@ -4293,7 +4290,7 @@
         <v>1</v>
       </c>
       <c r="M88" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>